<commit_message>
refactor(analisis): eliminar cod_cliente y razon_social de BD, API, interfaz y plantilla Excel
</commit_message>
<xml_diff>
--- a/modelo_importar_analisis.xlsx
+++ b/modelo_importar_analisis.xlsx
@@ -398,17 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:G4"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="17.83203125" customWidth="1"/>
-    <col min="7" max="7" width="17.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="19.83203125" customWidth="1"/>
+    <col min="7" max="7" width="19.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -433,12 +431,6 @@
       <c r="G1" t="str">
         <v>cantidad_motivo</v>
       </c>
-      <c r="H1" t="str">
-        <v>cod_cliente</v>
-      </c>
-      <c r="I1" t="str">
-        <v>razon_social</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -462,12 +454,6 @@
       <c r="G2">
         <v>3</v>
       </c>
-      <c r="H2" t="str">
-        <v>C00123</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Jorge Villasante</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -491,16 +477,10 @@
       <c r="G3">
         <v>2</v>
       </c>
-      <c r="H3" t="str">
-        <v>C00456</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Claudia Flores</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Ausente</v>
+        <v>Producto Defectuoso</v>
       </c>
       <c r="B4">
         <v>45.9</v>
@@ -520,23 +500,17 @@
       <c r="G4">
         <v>1</v>
       </c>
-      <c r="H4" t="str">
-        <v>C00123</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Jorge Villasante</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E8"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -681,43 +655,9 @@
         <v>Cantidad motivo (default 0)</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>cod_cliente</v>
-      </c>
-      <c r="B9" t="str">
-        <v>No</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Texto</v>
-      </c>
-      <c r="D9" t="str">
-        <v>C00123</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Código del cliente</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>razon_social</v>
-      </c>
-      <c r="B10" t="str">
-        <v>No</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Texto</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Jorge Villasante</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Razón social; se cuenta como cliente único</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>